<commit_message>
Full Top to Bottom Results Run
</commit_message>
<xml_diff>
--- a/results/Confusion_Matrix_Stats_Compare.xlsx
+++ b/results/Confusion_Matrix_Stats_Compare.xlsx
@@ -2228,7 +2228,7 @@
         <v>0.2145143665598397</v>
       </c>
       <c r="D19" t="n">
-        <v>0.1131478147964039</v>
+        <v>0.1131478147964038</v>
       </c>
       <c r="E19" t="n">
         <v>0.1048768519516965</v>
@@ -2240,7 +2240,7 @@
         <v>0.178728887534933</v>
       </c>
       <c r="H19" t="n">
-        <v>0.2437024876972061</v>
+        <v>0.243702487697206</v>
       </c>
       <c r="I19" t="n">
         <v>0.4451015891409608</v>
@@ -2285,10 +2285,10 @@
         <v>0.1373543897805134</v>
       </c>
       <c r="W19" t="n">
-        <v>0.1638683877678075</v>
+        <v>0.1638683877678074</v>
       </c>
       <c r="X19" t="n">
-        <v>0.2818104286150634</v>
+        <v>0.2818104286150633</v>
       </c>
       <c r="Y19" t="n">
         <v>0.5243960091673104</v>
@@ -2303,7 +2303,7 @@
         <v>0.1205711616688487</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.07961968039968984</v>
+        <v>0.07961968039968982</v>
       </c>
       <c r="AD19" t="n">
         <v>0.1193832105865548</v>
@@ -2315,7 +2315,7 @@
         <v>0.2559732612523407</v>
       </c>
       <c r="AG19" t="n">
-        <v>0.5423730220429928</v>
+        <v>0.5423730220429929</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Work On Results Section
</commit_message>
<xml_diff>
--- a/results/Confusion_Matrix_Stats_Compare.xlsx
+++ b/results/Confusion_Matrix_Stats_Compare.xlsx
@@ -2240,7 +2240,7 @@
         <v>0.178728887534933</v>
       </c>
       <c r="H19" t="n">
-        <v>0.243702487697206</v>
+        <v>0.2437024876972061</v>
       </c>
       <c r="I19" t="n">
         <v>0.4451015891409608</v>
@@ -2303,7 +2303,7 @@
         <v>0.1205711616688487</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.07961968039968982</v>
+        <v>0.07961968039968984</v>
       </c>
       <c r="AD19" t="n">
         <v>0.1193832105865548</v>
@@ -2315,7 +2315,7 @@
         <v>0.2559732612523407</v>
       </c>
       <c r="AG19" t="n">
-        <v>0.5423730220429929</v>
+        <v>0.5423730220429928</v>
       </c>
     </row>
   </sheetData>

</xml_diff>